<commit_message>
UPDATE: product and cart
</commit_message>
<xml_diff>
--- a/02_Test_Cases/TC_Module02_Cart_Product.xlsx
+++ b/02_Test_Cases/TC_Module02_Cart_Product.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\ktpm\manual_testing\02_Test_Cases\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6DB2D3-41CB-472D-B5EC-75530C6634A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,15 +24,436 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="101">
+  <si>
+    <t>TC_ID</t>
+  </si>
+  <si>
+    <t>Tiêu đề (Title)</t>
+  </si>
+  <si>
+    <t>Điều kiện trước</t>
+  </si>
+  <si>
+    <t>Các bước thực hiện</t>
+  </si>
+  <si>
+    <t>Kết quả mong đợi</t>
+  </si>
+  <si>
+    <t>Loại (Type)</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Tìm kiếm sản phẩm hợp lệ</t>
+  </si>
+  <si>
+    <t>Trang Products</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng sản phẩm "Blue Top".</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>TC_CART_004</t>
+  </si>
+  <si>
+    <t>Trang chi tiết</t>
+  </si>
+  <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>TC_CART_005</t>
+  </si>
+  <si>
+    <t>Nhập số lượng bằng 0</t>
+  </si>
+  <si>
+    <t>TC_CART_006</t>
+  </si>
+  <si>
+    <t>TC_CART_007</t>
+  </si>
+  <si>
+    <t>Trang chủ</t>
+  </si>
+  <si>
+    <t>TC_CART_008</t>
+  </si>
+  <si>
+    <t>TC_CART_009</t>
+  </si>
+  <si>
+    <t>Giỏ hàng</t>
+  </si>
+  <si>
+    <t>Giỏ hàng có 1 SP</t>
+  </si>
+  <si>
+    <t>TC_CART_012</t>
+  </si>
+  <si>
+    <t>TC_CART_013</t>
+  </si>
+  <si>
+    <t>TC_CART_014</t>
+  </si>
+  <si>
+    <t>Nhập chữ vào ô số lượng</t>
+  </si>
+  <si>
+    <t>TC_CART_016</t>
+  </si>
+  <si>
+    <t>TC_CART_017</t>
+  </si>
+  <si>
+    <t>TC_CART_020</t>
+  </si>
+  <si>
+    <t>Tìm kiếm sản phẩm không tồn tại</t>
+  </si>
+  <si>
+    <t>Hiển thị thông báo "No results found".</t>
+  </si>
+  <si>
+    <t>Tìm kiếm với chuỗi ký tự đặc biệt</t>
+  </si>
+  <si>
+    <t>Hệ thống không crash, hiển thị không tìm thấy kết quả.</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Nhập số lượng âm (-) tại trang chi tiết</t>
+  </si>
+  <si>
+    <t>Hệ thống không nhận giá trị âm hoặc báo lỗi.</t>
+  </si>
+  <si>
+    <t>Hệ thống không cho phép thêm 0 sản phẩm vào giỏ.</t>
+  </si>
+  <si>
+    <t>Nhập số lượng cực lớn (Max int)</t>
+  </si>
+  <si>
+    <t>Hệ thống hiển thị cảnh báo giới hạn số lượng đặt hàng.</t>
+  </si>
+  <si>
+    <t>Ô nhập tự động xóa chữ hoặc báo lỗi định dạng số.</t>
+  </si>
+  <si>
+    <t>Thêm sản phẩm khi chưa đăng nhập</t>
+  </si>
+  <si>
+    <t>1. Nhấn "Add to cart" tại một SP bất kỳ.</t>
+  </si>
+  <si>
+    <t>Hiển thị popup "Added!" thành công.</t>
+  </si>
+  <si>
+    <t>Xóa sản phẩm cuối cùng khỏi giỏ</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "X" tại sản phẩm.</t>
+  </si>
+  <si>
+    <t>Giỏ hàng trống, hiện thông báo "Cart is empty!".</t>
+  </si>
+  <si>
+    <t>Để trống ô Search và nhấn tìm</t>
+  </si>
+  <si>
+    <t>Không thực hiện tìm kiếm hoặc giữ nguyên danh sách.</t>
+  </si>
+  <si>
+    <t>Nhập Script tấn công vào ô Search</t>
+  </si>
+  <si>
+    <t>Hệ thống lọc script, không thực thi mã độc (XSS).</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Chỉnh sửa số lượng trong Cart thành số âm</t>
+  </si>
+  <si>
+    <t>1. Tại trang Cart, cố tình sửa Quantity thành -1.</t>
+  </si>
+  <si>
+    <t>Hệ thống tự động về 1 hoặc báo lỗi.</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính Read-only của thành tiền</t>
+  </si>
+  <si>
+    <t>1. Thử click và sửa ô "Total" của từng dòng SP.</t>
+  </si>
+  <si>
+    <t>Ô Total không cho phép sửa thủ công.</t>
+  </si>
+  <si>
+    <t>Thêm SP lặp lại nhiều lần</t>
+  </si>
+  <si>
+    <t>1. Nhấn "Add to cart" SP A liên tục 3 lần.</t>
+  </si>
+  <si>
+    <t>Quantity của SP A trong giỏ tăng lên 3.</t>
+  </si>
+  <si>
+    <t>Nhập khoảng trắng vào ô Search</t>
+  </si>
+  <si>
+    <t>Hệ thống xử lý như trường hợp để trống.</t>
+  </si>
+  <si>
+    <t>Checkout khi giỏ hàng đang trống</t>
+  </si>
+  <si>
+    <t>Giỏ hàng trống</t>
+  </si>
+  <si>
+    <t>Redirect về trang giỏ hàng hoặc báo lỗi giỏ trống.</t>
+  </si>
+  <si>
+    <t>Nhập số thập phân vào số lượng</t>
+  </si>
+  <si>
+    <t>Báo lỗi hoặc tự làm tròn thành số nguyên.</t>
+  </si>
+  <si>
+    <t>SQL Injection vào ô Search</t>
+  </si>
+  <si>
+    <t>Hệ thống xử lý an toàn, không lộ dữ liệu DB.</t>
+  </si>
+  <si>
+    <t>Thêm sản phẩm có Quantity là ký tự lạ</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Nhập các ký tự </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>!@#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> vào ô Quantity.</t>
+    </r>
+  </si>
+  <si>
+    <t>Hệ thống chặn không cho nhập hoặc báo lỗi.</t>
+  </si>
+  <si>
+    <t>Refresh trang khi đang thêm SP</t>
+  </si>
+  <si>
+    <t>1. Nhấn "Add to cart" và F5 ngay lập tức.</t>
+  </si>
+  <si>
+    <t>Giỏ hàng không bị lỗi dữ liệu hoặc SP chưa được thêm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Nhập "Blue Top" vào ô Search.
+2. Nhấn icon Search.
+</t>
+  </si>
+  <si>
+    <t>1. Nhập "Iphone 15" vào ô Search.
+2. Nhấn icon Search.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Nhập </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>@#$%^&amp;*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> vào ô Search.
+2. Nhấn icon Search.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Nhập "-5" vào ô Quantity.
+2. Nhấn "Add to cart".</t>
+  </si>
+  <si>
+    <t>1. Nhập "0" vào ô Quantity.
+2. Nhấn "Add to cart".</t>
+  </si>
+  <si>
+    <t>1. Nhập "999999" vào ô Quantity.
+2. Nhấn "Add to cart".</t>
+  </si>
+  <si>
+    <t>1. Nhập "abc" vào ô Quantity.
+2. Nhấn "Add to cart".</t>
+  </si>
+  <si>
+    <t>1. Không nhập gì vào ô Search.
+2. Nhấn icon Search.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Nhập </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.
+2. Nhấn Search.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Nhập " " (space) vào ô Search.
+2. Nhấn Search.</t>
+  </si>
+  <si>
+    <t>1. Cố tình truy cập URL /checkout.
+2. Nhấn thanh toán.</t>
+  </si>
+  <si>
+    <t>1. Nhập "1.5" vào ô Quantity.
+2. Nhấn "Add to cart".</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Nhập </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>' OR '1'='1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> vào ô Search.
+2. Nhấn Search.</t>
+    </r>
+  </si>
+  <si>
+    <t>TC_PRODUCT_001</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_002</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_003</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_010</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_011</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_015</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_018</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_019</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF444746"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +464,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -45,12 +472,52 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +797,503 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="34.88671875" customWidth="1"/>
+    <col min="3" max="3" width="35.88671875" customWidth="1"/>
+    <col min="4" max="4" width="30.44140625" customWidth="1"/>
+    <col min="5" max="5" width="38.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="14.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="15" thickBot="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="43.8" customHeight="1" thickBot="1">
+      <c r="A2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="43.2" customHeight="1" thickBot="1">
+      <c r="A3" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="50.4" customHeight="1" thickBot="1">
+      <c r="A4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="39" customHeight="1" thickBot="1">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="52.2" customHeight="1" thickBot="1">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="60" customHeight="1" thickBot="1">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="59.4" customHeight="1" thickBot="1">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="46.8" customHeight="1" thickBot="1">
+      <c r="A9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="54" customHeight="1" thickBot="1">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="51.6" customHeight="1" thickBot="1">
+      <c r="A11" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="57" customHeight="1" thickBot="1">
+      <c r="A12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="48.6" customHeight="1" thickBot="1">
+      <c r="A13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="48.6" customHeight="1" thickBot="1">
+      <c r="A14" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="46.2" customHeight="1">
+      <c r="A15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="64.8" customHeight="1" thickBot="1">
+      <c r="A16" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="63" customHeight="1" thickBot="1">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="48.6" customHeight="1" thickBot="1">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="60.6" customHeight="1" thickBot="1">
+      <c r="A19" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="39" customHeight="1" thickBot="1">
+      <c r="A20" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="42.6" customHeight="1" thickBot="1">
+      <c r="A21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>